<commit_message>
feat: adequacao e doc da planilha modelo
</commit_message>
<xml_diff>
--- a/modelo-razao-importacao.xlsx
+++ b/modelo-razao-importacao.xlsx
@@ -539,9 +539,9 @@
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -559,7 +559,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>CENTRO DE ESTETICA GRANJA VIANA LTDA</t>
+          <t>EMPRESA MODELO LTDA</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>12.795.276/0001-92</t>
+          <t>11.222.333/0001-81</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>saldo_exercicio</t>
+          <t>saldo_exercicio_original</t>
         </is>
       </c>
     </row>
@@ -711,17 +711,17 @@
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Valor a debito, se houver</t>
+          <t>Valor a debito, se houver; preencha debito ou credito, nunca ambos.</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Valor a credito, se houver</t>
+          <t>Valor a credito, se houver; preencha debito ou credito, nunca ambos.</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>Saldo informado pelo relatorio, opcional</t>
+          <t>Saldo do relatorio, opcional e apenas para conferencia. Ex: 1156,68C</t>
         </is>
       </c>
     </row>
@@ -742,12 +742,12 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>CAIXA</t>
+          <t>CAIXA MODELO</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>PAGTO.PRO-LABORE.REF.</t>
+          <t>PAGAMENTO FORNECEDOR MODELO</t>
         </is>
       </c>
       <c r="G12" s="10" t="n">
@@ -757,8 +757,10 @@
       <c r="I12" s="11" t="n">
         <v>1256.68</v>
       </c>
-      <c r="J12" s="11" t="n">
-        <v>-1156.68</v>
+      <c r="J12" s="11" t="inlineStr">
+        <is>
+          <t>1156,68C</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -778,12 +780,12 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>CAIXA</t>
+          <t>CAIXA MODELO</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>PAGTO.FERIAS DO FUNC.</t>
+          <t>PAGAMENTO FERIAS MODELO</t>
         </is>
       </c>
       <c r="G13" s="10" t="n">
@@ -793,8 +795,10 @@
       <c r="I13" s="11" t="n">
         <v>185</v>
       </c>
-      <c r="J13" s="11" t="n">
-        <v>-1341.68</v>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>1341,68C</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -814,23 +818,25 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>CAIXA</t>
+          <t>CAIXA MODELO</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>PAGTO.PRO-LABORE.REF.</t>
+          <t>RECEBIMENTO CLIENTE MODELO</t>
         </is>
       </c>
       <c r="G14" s="10" t="n">
         <v>20951</v>
       </c>
-      <c r="H14" s="11" t="n"/>
-      <c r="I14" s="11" t="n">
-        <v>1256.68</v>
-      </c>
-      <c r="J14" s="11" t="n">
-        <v>-2598.36</v>
+      <c r="H14" s="11" t="n">
+        <v>500</v>
+      </c>
+      <c r="I14" s="11" t="n"/>
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>841,68C</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -2005,7 +2011,7 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Cada linha deve ter debito OU credito preenchido. Nao preencha os dois na mesma linha.</t>
+          <t>Cada linha deve ter debito ou credito preenchido. Nao preencha os dois na mesma linha.</t>
         </is>
       </c>
       <c r="C115" s="5" t="n"/>
@@ -2035,10 +2041,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2051,35 +2057,35 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>1. Preencha Empresa, CNPJ e periodo no topo da aba Razao.</t>
+          <t>1. Preencha Empresa, CNPJ, Periodo inicio e Periodo fim no topo da aba Razao.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>2. Copie os lancamentos do relatorio original para a tabela a partir da linha 12.</t>
+          <t>2. Copie ou digite os lancamentos na tabela a partir da linha 12.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>3. Use conta_origem para o codigo da conta do bloco Conta:.</t>
+          <t>3. Use conta_origem para o codigo reduzido da conta do bloco Conta:.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>4. Use contrapartida para a coluna Cta.C.Part. do relatorio original.</t>
+          <t>4. Use contrapartida para a conta equivalente a Cta.C.Part. do relatorio original.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>5. Preencha apenas debito ou credito por linha.</t>
+          <t>5. Preencha apenas debito ou credito por linha. Nunca preencha os dois.</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2099,14 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>7. Se o CNPJ corresponder a uma empresa inativa, o importador deve bloquear a importacao.</t>
+          <t>7. saldo_exercicio_original e opcional, serve apenas para conferencia e nao define debito/credito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>8. Nao informe cod_dominio neste modelo. A importacao nao cria empresa automaticamente.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: adequacao e doc da planilha modelo (#178)
</commit_message>
<xml_diff>
--- a/modelo-razao-importacao.xlsx
+++ b/modelo-razao-importacao.xlsx
@@ -539,9 +539,9 @@
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -559,7 +559,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>CENTRO DE ESTETICA GRANJA VIANA LTDA</t>
+          <t>EMPRESA MODELO LTDA</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>12.795.276/0001-92</t>
+          <t>11.222.333/0001-81</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>saldo_exercicio</t>
+          <t>saldo_exercicio_original</t>
         </is>
       </c>
     </row>
@@ -711,17 +711,17 @@
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Valor a debito, se houver</t>
+          <t>Valor a debito, se houver; preencha debito ou credito, nunca ambos.</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Valor a credito, se houver</t>
+          <t>Valor a credito, se houver; preencha debito ou credito, nunca ambos.</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>Saldo informado pelo relatorio, opcional</t>
+          <t>Saldo do relatorio, opcional e apenas para conferencia. Ex: 1156,68C</t>
         </is>
       </c>
     </row>
@@ -742,12 +742,12 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>CAIXA</t>
+          <t>CAIXA MODELO</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>PAGTO.PRO-LABORE.REF.</t>
+          <t>PAGAMENTO FORNECEDOR MODELO</t>
         </is>
       </c>
       <c r="G12" s="10" t="n">
@@ -757,8 +757,10 @@
       <c r="I12" s="11" t="n">
         <v>1256.68</v>
       </c>
-      <c r="J12" s="11" t="n">
-        <v>-1156.68</v>
+      <c r="J12" s="11" t="inlineStr">
+        <is>
+          <t>1156,68C</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -778,12 +780,12 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>CAIXA</t>
+          <t>CAIXA MODELO</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>PAGTO.FERIAS DO FUNC.</t>
+          <t>PAGAMENTO FERIAS MODELO</t>
         </is>
       </c>
       <c r="G13" s="10" t="n">
@@ -793,8 +795,10 @@
       <c r="I13" s="11" t="n">
         <v>185</v>
       </c>
-      <c r="J13" s="11" t="n">
-        <v>-1341.68</v>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>1341,68C</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -814,23 +818,25 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>CAIXA</t>
+          <t>CAIXA MODELO</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>PAGTO.PRO-LABORE.REF.</t>
+          <t>RECEBIMENTO CLIENTE MODELO</t>
         </is>
       </c>
       <c r="G14" s="10" t="n">
         <v>20951</v>
       </c>
-      <c r="H14" s="11" t="n"/>
-      <c r="I14" s="11" t="n">
-        <v>1256.68</v>
-      </c>
-      <c r="J14" s="11" t="n">
-        <v>-2598.36</v>
+      <c r="H14" s="11" t="n">
+        <v>500</v>
+      </c>
+      <c r="I14" s="11" t="n"/>
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>841,68C</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -2005,7 +2011,7 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Cada linha deve ter debito OU credito preenchido. Nao preencha os dois na mesma linha.</t>
+          <t>Cada linha deve ter debito ou credito preenchido. Nao preencha os dois na mesma linha.</t>
         </is>
       </c>
       <c r="C115" s="5" t="n"/>
@@ -2035,10 +2041,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2051,35 +2057,35 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>1. Preencha Empresa, CNPJ e periodo no topo da aba Razao.</t>
+          <t>1. Preencha Empresa, CNPJ, Periodo inicio e Periodo fim no topo da aba Razao.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>2. Copie os lancamentos do relatorio original para a tabela a partir da linha 12.</t>
+          <t>2. Copie ou digite os lancamentos na tabela a partir da linha 12.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>3. Use conta_origem para o codigo da conta do bloco Conta:.</t>
+          <t>3. Use conta_origem para o codigo reduzido da conta do bloco Conta:.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>4. Use contrapartida para a coluna Cta.C.Part. do relatorio original.</t>
+          <t>4. Use contrapartida para a conta equivalente a Cta.C.Part. do relatorio original.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>5. Preencha apenas debito ou credito por linha.</t>
+          <t>5. Preencha apenas debito ou credito por linha. Nunca preencha os dois.</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2099,14 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>7. Se o CNPJ corresponder a uma empresa inativa, o importador deve bloquear a importacao.</t>
+          <t>7. saldo_exercicio_original e opcional, serve apenas para conferencia e nao define debito/credito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>8. Nao informe cod_dominio neste modelo. A importacao nao cria empresa automaticamente.</t>
         </is>
       </c>
     </row>

</xml_diff>